<commit_message>
Remove FRCoreValueSetEncounterClass binding, add common codes as examples in class.short
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> ca3c959b33988fc60a1cbc080c252b0dad7d4c61
</commit_message>
<xml_diff>
--- a/nr-doc-core-encounter/ig/StructureDefinition-fr-core-encounter.xlsx
+++ b/nr-doc-core-encounter/ig/StructureDefinition-fr-core-encounter.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3607" uniqueCount="575">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3608" uniqueCount="574">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-29T12:39:39+00:00</t>
+    <t>2026-07-21T11:52:46+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -943,13 +943,22 @@
     <t>Encounter.class</t>
   </si>
   <si>
-    <t>Type de rencontre (codes HL7 ActEncounterCode ou codes spécifiques aux cas d'usages)</t>
+    <t>Type de rencontre (codes HL7 ActEncounterCode ou codes spécifiques aux cas d'usages)
+Exemples de codes les plus courants (http://terminology.hl7.org/CodeSystem/v3-ActCode) :
+- ACUTE : Inpatient acute
+- NONAC : Inpatient non acute
+- PRENC : Pre-admission
+- SS : Short stay
+- VR : Virtual</t>
   </si>
   <si>
     <t>Concepts representing classification of patient encounter such as ambulatory (outpatient), inpatient, emergency, home health or others due to local variations.</t>
   </si>
   <si>
-    <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-encounter-class|2.2.0</t>
+    <t>Classification of the encounter.</t>
+  </si>
+  <si>
+    <t>http://terminology.hl7.org/ValueSet/v3-ActEncounterCode|3.0.0</t>
   </si>
   <si>
     <t>.inboundRelationship[typeCode=SUBJ].source[classCode=LIST].code</t>
@@ -986,12 +995,6 @@
   </si>
   <si>
     <t>inpatient | outpatient | ambulatory | emergency +.</t>
-  </si>
-  <si>
-    <t>Classification of the encounter.</t>
-  </si>
-  <si>
-    <t>http://terminology.hl7.org/ValueSet/v3-ActEncounterCode|3.0.0</t>
   </si>
   <si>
     <t>Encounter.classHistory.period</t>
@@ -1541,7 +1544,7 @@
     <t>From where patient was admitted (physician referral, transfer).</t>
   </si>
   <si>
-    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-modalite-entree-cisis|20260420150251</t>
+    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-modalite-entree-cisis|20260619134043</t>
   </si>
   <si>
     <t>.admissionReferralSourceCode</t>
@@ -6316,9 +6319,11 @@
       <c r="X37" t="s" s="2">
         <v>152</v>
       </c>
-      <c r="Y37" s="2"/>
+      <c r="Y37" t="s" s="2">
+        <v>300</v>
+      </c>
       <c r="Z37" t="s" s="2">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="AA37" t="s" s="2">
         <v>81</v>
@@ -6354,21 +6359,21 @@
         <v>81</v>
       </c>
       <c r="AL37" t="s" s="2">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="AM37" t="s" s="2">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="AN37" t="s" s="2">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -6394,10 +6399,10 @@
         <v>281</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
@@ -6448,7 +6453,7 @@
         <v>81</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>79</v>
@@ -6477,10 +6482,10 @@
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -6589,10 +6594,10 @@
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -6703,10 +6708,10 @@
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6819,10 +6824,10 @@
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -6848,10 +6853,10 @@
         <v>148</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
@@ -6881,10 +6886,10 @@
         <v>152</v>
       </c>
       <c r="Y42" t="s" s="2">
-        <v>313</v>
+        <v>300</v>
       </c>
       <c r="Z42" t="s" s="2">
-        <v>314</v>
+        <v>301</v>
       </c>
       <c r="AA42" t="s" s="2">
         <v>81</v>
@@ -6902,7 +6907,7 @@
         <v>81</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>89</v>
@@ -6931,10 +6936,10 @@
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -6960,10 +6965,10 @@
         <v>256</v>
       </c>
       <c r="L43" t="s" s="2">
+        <v>315</v>
+      </c>
+      <c r="M43" t="s" s="2">
         <v>316</v>
-      </c>
-      <c r="M43" t="s" s="2">
-        <v>317</v>
       </c>
       <c r="N43" s="2"/>
       <c r="O43" s="2"/>
@@ -7014,7 +7019,7 @@
         <v>81</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>89</v>
@@ -7043,10 +7048,10 @@
     </row>
     <row r="44">
       <c r="A44" t="s" s="2">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -7072,13 +7077,13 @@
         <v>230</v>
       </c>
       <c r="L44" t="s" s="2">
+        <v>318</v>
+      </c>
+      <c r="M44" t="s" s="2">
         <v>319</v>
       </c>
-      <c r="M44" t="s" s="2">
+      <c r="N44" t="s" s="2">
         <v>320</v>
-      </c>
-      <c r="N44" t="s" s="2">
-        <v>321</v>
       </c>
       <c r="O44" s="2"/>
       <c r="P44" t="s" s="2">
@@ -7108,7 +7113,7 @@
       </c>
       <c r="Y44" s="2"/>
       <c r="Z44" t="s" s="2">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="AA44" t="s" s="2">
         <v>81</v>
@@ -7126,7 +7131,7 @@
         <v>81</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>79</v>
@@ -7141,24 +7146,24 @@
         <v>101</v>
       </c>
       <c r="AK44" t="s" s="2">
+        <v>322</v>
+      </c>
+      <c r="AL44" t="s" s="2">
         <v>323</v>
       </c>
-      <c r="AL44" t="s" s="2">
+      <c r="AM44" t="s" s="2">
+        <v>303</v>
+      </c>
+      <c r="AN44" t="s" s="2">
         <v>324</v>
-      </c>
-      <c r="AM44" t="s" s="2">
-        <v>302</v>
-      </c>
-      <c r="AN44" t="s" s="2">
-        <v>325</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -7184,10 +7189,10 @@
         <v>230</v>
       </c>
       <c r="L45" t="s" s="2">
+        <v>326</v>
+      </c>
+      <c r="M45" t="s" s="2">
         <v>327</v>
-      </c>
-      <c r="M45" t="s" s="2">
-        <v>328</v>
       </c>
       <c r="N45" s="2"/>
       <c r="O45" s="2"/>
@@ -7217,11 +7222,11 @@
         <v>160</v>
       </c>
       <c r="Y45" t="s" s="2">
+        <v>328</v>
+      </c>
+      <c r="Z45" t="s" s="2">
         <v>329</v>
       </c>
-      <c r="Z45" t="s" s="2">
-        <v>330</v>
-      </c>
       <c r="AA45" t="s" s="2">
         <v>81</v>
       </c>
@@ -7238,7 +7243,7 @@
         <v>81</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>79</v>
@@ -7253,7 +7258,7 @@
         <v>101</v>
       </c>
       <c r="AK45" t="s" s="2">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="AL45" t="s" s="2">
         <v>107</v>
@@ -7262,15 +7267,15 @@
         <v>81</v>
       </c>
       <c r="AN45" t="s" s="2">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s" s="2">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -7296,10 +7301,10 @@
         <v>230</v>
       </c>
       <c r="L46" t="s" s="2">
+        <v>332</v>
+      </c>
+      <c r="M46" t="s" s="2">
         <v>333</v>
-      </c>
-      <c r="M46" t="s" s="2">
-        <v>334</v>
       </c>
       <c r="N46" s="2"/>
       <c r="O46" s="2"/>
@@ -7329,11 +7334,11 @@
         <v>160</v>
       </c>
       <c r="Y46" t="s" s="2">
+        <v>333</v>
+      </c>
+      <c r="Z46" t="s" s="2">
         <v>334</v>
       </c>
-      <c r="Z46" t="s" s="2">
-        <v>335</v>
-      </c>
       <c r="AA46" t="s" s="2">
         <v>81</v>
       </c>
@@ -7350,7 +7355,7 @@
         <v>81</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>79</v>
@@ -7368,25 +7373,25 @@
         <v>81</v>
       </c>
       <c r="AL46" t="s" s="2">
+        <v>335</v>
+      </c>
+      <c r="AM46" t="s" s="2">
         <v>336</v>
       </c>
-      <c r="AM46" t="s" s="2">
+      <c r="AN46" t="s" s="2">
         <v>337</v>
-      </c>
-      <c r="AN46" t="s" s="2">
-        <v>338</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="2">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="E47" s="2"/>
       <c r="F47" t="s" s="2">
@@ -7405,16 +7410,16 @@
         <v>90</v>
       </c>
       <c r="K47" t="s" s="2">
+        <v>340</v>
+      </c>
+      <c r="L47" t="s" s="2">
         <v>341</v>
       </c>
-      <c r="L47" t="s" s="2">
+      <c r="M47" t="s" s="2">
         <v>342</v>
       </c>
-      <c r="M47" t="s" s="2">
+      <c r="N47" t="s" s="2">
         <v>343</v>
-      </c>
-      <c r="N47" t="s" s="2">
-        <v>344</v>
       </c>
       <c r="O47" s="2"/>
       <c r="P47" t="s" s="2">
@@ -7464,7 +7469,7 @@
         <v>81</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>79</v>
@@ -7479,24 +7484,24 @@
         <v>101</v>
       </c>
       <c r="AK47" t="s" s="2">
+        <v>344</v>
+      </c>
+      <c r="AL47" t="s" s="2">
         <v>345</v>
       </c>
-      <c r="AL47" t="s" s="2">
+      <c r="AM47" t="s" s="2">
         <v>346</v>
       </c>
-      <c r="AM47" t="s" s="2">
+      <c r="AN47" t="s" s="2">
         <v>347</v>
-      </c>
-      <c r="AN47" t="s" s="2">
-        <v>348</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s" s="2">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -7519,13 +7524,13 @@
         <v>90</v>
       </c>
       <c r="K48" t="s" s="2">
+        <v>349</v>
+      </c>
+      <c r="L48" t="s" s="2">
         <v>350</v>
       </c>
-      <c r="L48" t="s" s="2">
+      <c r="M48" t="s" s="2">
         <v>351</v>
-      </c>
-      <c r="M48" t="s" s="2">
-        <v>352</v>
       </c>
       <c r="N48" s="2"/>
       <c r="O48" s="2"/>
@@ -7576,7 +7581,7 @@
         <v>81</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>79</v>
@@ -7591,28 +7596,28 @@
         <v>101</v>
       </c>
       <c r="AK48" t="s" s="2">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="AL48" t="s" s="2">
         <v>107</v>
       </c>
       <c r="AM48" t="s" s="2">
+        <v>353</v>
+      </c>
+      <c r="AN48" t="s" s="2">
         <v>354</v>
-      </c>
-      <c r="AN48" t="s" s="2">
-        <v>355</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s" s="2">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E49" s="2"/>
       <c r="F49" t="s" s="2">
@@ -7631,13 +7636,13 @@
         <v>81</v>
       </c>
       <c r="K49" t="s" s="2">
+        <v>357</v>
+      </c>
+      <c r="L49" t="s" s="2">
         <v>358</v>
       </c>
-      <c r="L49" t="s" s="2">
+      <c r="M49" t="s" s="2">
         <v>359</v>
-      </c>
-      <c r="M49" t="s" s="2">
-        <v>360</v>
       </c>
       <c r="N49" s="2"/>
       <c r="O49" s="2"/>
@@ -7688,7 +7693,7 @@
         <v>81</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>79</v>
@@ -7703,10 +7708,10 @@
         <v>101</v>
       </c>
       <c r="AK49" t="s" s="2">
+        <v>360</v>
+      </c>
+      <c r="AL49" t="s" s="2">
         <v>361</v>
-      </c>
-      <c r="AL49" t="s" s="2">
-        <v>362</v>
       </c>
       <c r="AM49" t="s" s="2">
         <v>81</v>
@@ -7717,10 +7722,10 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -7746,10 +7751,10 @@
         <v>281</v>
       </c>
       <c r="L50" t="s" s="2">
+        <v>363</v>
+      </c>
+      <c r="M50" t="s" s="2">
         <v>364</v>
-      </c>
-      <c r="M50" t="s" s="2">
-        <v>365</v>
       </c>
       <c r="N50" s="2"/>
       <c r="O50" s="2"/>
@@ -7800,7 +7805,7 @@
         <v>81</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>79</v>
@@ -7815,24 +7820,24 @@
         <v>101</v>
       </c>
       <c r="AK50" t="s" s="2">
+        <v>365</v>
+      </c>
+      <c r="AL50" t="s" s="2">
         <v>366</v>
       </c>
-      <c r="AL50" t="s" s="2">
+      <c r="AM50" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN50" t="s" s="2">
         <v>367</v>
-      </c>
-      <c r="AM50" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AN50" t="s" s="2">
-        <v>368</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s" s="2">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -7941,10 +7946,10 @@
     </row>
     <row r="52">
       <c r="A52" t="s" s="2">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -8055,10 +8060,10 @@
     </row>
     <row r="53">
       <c r="A53" t="s" s="2">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -8171,10 +8176,10 @@
     </row>
     <row r="54">
       <c r="A54" t="s" s="2">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -8200,13 +8205,13 @@
         <v>230</v>
       </c>
       <c r="L54" t="s" s="2">
+        <v>372</v>
+      </c>
+      <c r="M54" t="s" s="2">
         <v>373</v>
       </c>
-      <c r="M54" t="s" s="2">
+      <c r="N54" t="s" s="2">
         <v>374</v>
-      </c>
-      <c r="N54" t="s" s="2">
-        <v>375</v>
       </c>
       <c r="O54" s="2"/>
       <c r="P54" t="s" s="2">
@@ -8235,10 +8240,10 @@
         <v>152</v>
       </c>
       <c r="Y54" t="s" s="2">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="Z54" t="s" s="2">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="AA54" t="s" s="2">
         <v>81</v>
@@ -8256,7 +8261,7 @@
         <v>81</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>79</v>
@@ -8271,24 +8276,24 @@
         <v>101</v>
       </c>
       <c r="AK54" t="s" s="2">
+        <v>376</v>
+      </c>
+      <c r="AL54" t="s" s="2">
         <v>377</v>
       </c>
-      <c r="AL54" t="s" s="2">
+      <c r="AM54" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN54" t="s" s="2">
         <v>378</v>
-      </c>
-      <c r="AM54" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AN54" t="s" s="2">
-        <v>379</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s" s="2">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -8314,10 +8319,10 @@
         <v>256</v>
       </c>
       <c r="L55" t="s" s="2">
+        <v>380</v>
+      </c>
+      <c r="M55" t="s" s="2">
         <v>381</v>
-      </c>
-      <c r="M55" t="s" s="2">
-        <v>382</v>
       </c>
       <c r="N55" s="2"/>
       <c r="O55" s="2"/>
@@ -8368,7 +8373,7 @@
         <v>81</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>79</v>
@@ -8386,21 +8391,21 @@
         <v>81</v>
       </c>
       <c r="AL55" t="s" s="2">
+        <v>382</v>
+      </c>
+      <c r="AM55" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN55" t="s" s="2">
         <v>383</v>
-      </c>
-      <c r="AM55" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AN55" t="s" s="2">
-        <v>384</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s" s="2">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
@@ -8423,13 +8428,13 @@
         <v>90</v>
       </c>
       <c r="K56" t="s" s="2">
+        <v>385</v>
+      </c>
+      <c r="L56" t="s" s="2">
         <v>386</v>
       </c>
-      <c r="L56" t="s" s="2">
+      <c r="M56" t="s" s="2">
         <v>387</v>
-      </c>
-      <c r="M56" t="s" s="2">
-        <v>388</v>
       </c>
       <c r="N56" s="2"/>
       <c r="O56" s="2"/>
@@ -8480,7 +8485,7 @@
         <v>81</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>79</v>
@@ -8495,24 +8500,24 @@
         <v>101</v>
       </c>
       <c r="AK56" t="s" s="2">
+        <v>388</v>
+      </c>
+      <c r="AL56" t="s" s="2">
         <v>389</v>
       </c>
-      <c r="AL56" t="s" s="2">
+      <c r="AM56" t="s" s="2">
         <v>390</v>
       </c>
-      <c r="AM56" t="s" s="2">
+      <c r="AN56" t="s" s="2">
         <v>391</v>
-      </c>
-      <c r="AN56" t="s" s="2">
-        <v>392</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s" s="2">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -8535,13 +8540,13 @@
         <v>90</v>
       </c>
       <c r="K57" t="s" s="2">
+        <v>393</v>
+      </c>
+      <c r="L57" t="s" s="2">
         <v>394</v>
       </c>
-      <c r="L57" t="s" s="2">
+      <c r="M57" t="s" s="2">
         <v>395</v>
-      </c>
-      <c r="M57" t="s" s="2">
-        <v>396</v>
       </c>
       <c r="N57" s="2"/>
       <c r="O57" s="2"/>
@@ -8592,7 +8597,7 @@
         <v>81</v>
       </c>
       <c r="AF57" t="s" s="2">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="AG57" t="s" s="2">
         <v>79</v>
@@ -8607,24 +8612,24 @@
         <v>101</v>
       </c>
       <c r="AK57" t="s" s="2">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="AL57" t="s" s="2">
+        <v>396</v>
+      </c>
+      <c r="AM57" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN57" t="s" s="2">
         <v>397</v>
-      </c>
-      <c r="AM57" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AN57" t="s" s="2">
-        <v>398</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s" s="2">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
@@ -8650,13 +8655,13 @@
         <v>256</v>
       </c>
       <c r="L58" t="s" s="2">
+        <v>399</v>
+      </c>
+      <c r="M58" t="s" s="2">
         <v>400</v>
       </c>
-      <c r="M58" t="s" s="2">
+      <c r="N58" t="s" s="2">
         <v>401</v>
-      </c>
-      <c r="N58" t="s" s="2">
-        <v>402</v>
       </c>
       <c r="O58" s="2"/>
       <c r="P58" t="s" s="2">
@@ -8706,7 +8711,7 @@
         <v>81</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>79</v>
@@ -8721,24 +8726,24 @@
         <v>101</v>
       </c>
       <c r="AK58" t="s" s="2">
+        <v>402</v>
+      </c>
+      <c r="AL58" t="s" s="2">
         <v>403</v>
       </c>
-      <c r="AL58" t="s" s="2">
+      <c r="AM58" t="s" s="2">
         <v>404</v>
       </c>
-      <c r="AM58" t="s" s="2">
+      <c r="AN58" t="s" s="2">
         <v>405</v>
-      </c>
-      <c r="AN58" t="s" s="2">
-        <v>406</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s" s="2">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -8761,16 +8766,16 @@
         <v>81</v>
       </c>
       <c r="K59" t="s" s="2">
+        <v>407</v>
+      </c>
+      <c r="L59" t="s" s="2">
         <v>408</v>
       </c>
-      <c r="L59" t="s" s="2">
+      <c r="M59" t="s" s="2">
         <v>409</v>
       </c>
-      <c r="M59" t="s" s="2">
+      <c r="N59" t="s" s="2">
         <v>410</v>
-      </c>
-      <c r="N59" t="s" s="2">
-        <v>411</v>
       </c>
       <c r="O59" s="2"/>
       <c r="P59" t="s" s="2">
@@ -8820,7 +8825,7 @@
         <v>81</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>79</v>
@@ -8835,28 +8840,28 @@
         <v>101</v>
       </c>
       <c r="AK59" t="s" s="2">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="AL59" t="s" s="2">
+        <v>411</v>
+      </c>
+      <c r="AM59" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN59" t="s" s="2">
         <v>412</v>
-      </c>
-      <c r="AM59" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AN59" t="s" s="2">
-        <v>413</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s" s="2">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="E60" s="2"/>
       <c r="F60" t="s" s="2">
@@ -8878,13 +8883,13 @@
         <v>230</v>
       </c>
       <c r="L60" t="s" s="2">
+        <v>415</v>
+      </c>
+      <c r="M60" t="s" s="2">
         <v>416</v>
       </c>
-      <c r="M60" t="s" s="2">
+      <c r="N60" t="s" s="2">
         <v>417</v>
-      </c>
-      <c r="N60" t="s" s="2">
-        <v>418</v>
       </c>
       <c r="O60" s="2"/>
       <c r="P60" t="s" s="2">
@@ -8913,11 +8918,11 @@
         <v>174</v>
       </c>
       <c r="Y60" t="s" s="2">
+        <v>418</v>
+      </c>
+      <c r="Z60" t="s" s="2">
         <v>419</v>
       </c>
-      <c r="Z60" t="s" s="2">
-        <v>420</v>
-      </c>
       <c r="AA60" t="s" s="2">
         <v>81</v>
       </c>
@@ -8934,7 +8939,7 @@
         <v>81</v>
       </c>
       <c r="AF60" t="s" s="2">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="AG60" t="s" s="2">
         <v>79</v>
@@ -8949,28 +8954,28 @@
         <v>101</v>
       </c>
       <c r="AK60" t="s" s="2">
+        <v>420</v>
+      </c>
+      <c r="AL60" t="s" s="2">
         <v>421</v>
       </c>
-      <c r="AL60" t="s" s="2">
+      <c r="AM60" t="s" s="2">
         <v>422</v>
       </c>
-      <c r="AM60" t="s" s="2">
+      <c r="AN60" t="s" s="2">
         <v>423</v>
-      </c>
-      <c r="AN60" t="s" s="2">
-        <v>424</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s" s="2">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="E61" s="2"/>
       <c r="F61" t="s" s="2">
@@ -8989,16 +8994,16 @@
         <v>90</v>
       </c>
       <c r="K61" t="s" s="2">
+        <v>425</v>
+      </c>
+      <c r="L61" t="s" s="2">
         <v>426</v>
       </c>
-      <c r="L61" t="s" s="2">
-        <v>427</v>
-      </c>
       <c r="M61" t="s" s="2">
+        <v>416</v>
+      </c>
+      <c r="N61" t="s" s="2">
         <v>417</v>
-      </c>
-      <c r="N61" t="s" s="2">
-        <v>418</v>
       </c>
       <c r="O61" s="2"/>
       <c r="P61" t="s" s="2">
@@ -9048,7 +9053,7 @@
         <v>81</v>
       </c>
       <c r="AF61" t="s" s="2">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="AG61" t="s" s="2">
         <v>79</v>
@@ -9063,24 +9068,24 @@
         <v>101</v>
       </c>
       <c r="AK61" t="s" s="2">
+        <v>420</v>
+      </c>
+      <c r="AL61" t="s" s="2">
         <v>421</v>
       </c>
-      <c r="AL61" t="s" s="2">
+      <c r="AM61" t="s" s="2">
         <v>422</v>
       </c>
-      <c r="AM61" t="s" s="2">
+      <c r="AN61" t="s" s="2">
         <v>423</v>
-      </c>
-      <c r="AN61" t="s" s="2">
-        <v>424</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="s" s="2">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -9106,10 +9111,10 @@
         <v>281</v>
       </c>
       <c r="L62" t="s" s="2">
+        <v>428</v>
+      </c>
+      <c r="M62" t="s" s="2">
         <v>429</v>
-      </c>
-      <c r="M62" t="s" s="2">
-        <v>430</v>
       </c>
       <c r="N62" s="2"/>
       <c r="O62" s="2"/>
@@ -9160,7 +9165,7 @@
         <v>81</v>
       </c>
       <c r="AF62" t="s" s="2">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="AG62" t="s" s="2">
         <v>79</v>
@@ -9178,7 +9183,7 @@
         <v>81</v>
       </c>
       <c r="AL62" t="s" s="2">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="AM62" t="s" s="2">
         <v>81</v>
@@ -9189,10 +9194,10 @@
     </row>
     <row r="63">
       <c r="A63" t="s" s="2">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
@@ -9301,10 +9306,10 @@
     </row>
     <row r="64">
       <c r="A64" t="s" s="2">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -9415,10 +9420,10 @@
     </row>
     <row r="65">
       <c r="A65" t="s" s="2">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" t="s" s="2">
@@ -9531,14 +9536,14 @@
     </row>
     <row r="66">
       <c r="A66" t="s" s="2">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" t="s" s="2">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="E66" s="2"/>
       <c r="F66" t="s" s="2">
@@ -9557,16 +9562,16 @@
         <v>90</v>
       </c>
       <c r="K66" t="s" s="2">
+        <v>436</v>
+      </c>
+      <c r="L66" t="s" s="2">
         <v>437</v>
       </c>
-      <c r="L66" t="s" s="2">
+      <c r="M66" t="s" s="2">
         <v>438</v>
       </c>
-      <c r="M66" t="s" s="2">
-        <v>439</v>
-      </c>
       <c r="N66" t="s" s="2">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="O66" s="2"/>
       <c r="P66" t="s" s="2">
@@ -9616,7 +9621,7 @@
         <v>81</v>
       </c>
       <c r="AF66" t="s" s="2">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="AG66" t="s" s="2">
         <v>89</v>
@@ -9631,24 +9636,24 @@
         <v>101</v>
       </c>
       <c r="AK66" t="s" s="2">
+        <v>439</v>
+      </c>
+      <c r="AL66" t="s" s="2">
         <v>440</v>
       </c>
-      <c r="AL66" t="s" s="2">
+      <c r="AM66" t="s" s="2">
+        <v>422</v>
+      </c>
+      <c r="AN66" t="s" s="2">
         <v>441</v>
-      </c>
-      <c r="AM66" t="s" s="2">
-        <v>423</v>
-      </c>
-      <c r="AN66" t="s" s="2">
-        <v>442</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="s" s="2">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" t="s" s="2">
@@ -9674,10 +9679,10 @@
         <v>230</v>
       </c>
       <c r="L67" t="s" s="2">
+        <v>443</v>
+      </c>
+      <c r="M67" t="s" s="2">
         <v>444</v>
-      </c>
-      <c r="M67" t="s" s="2">
-        <v>445</v>
       </c>
       <c r="N67" s="2"/>
       <c r="O67" s="2"/>
@@ -9707,11 +9712,11 @@
         <v>174</v>
       </c>
       <c r="Y67" t="s" s="2">
+        <v>445</v>
+      </c>
+      <c r="Z67" t="s" s="2">
         <v>446</v>
       </c>
-      <c r="Z67" t="s" s="2">
-        <v>447</v>
-      </c>
       <c r="AA67" t="s" s="2">
         <v>81</v>
       </c>
@@ -9728,7 +9733,7 @@
         <v>81</v>
       </c>
       <c r="AF67" t="s" s="2">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="AG67" t="s" s="2">
         <v>79</v>
@@ -9757,10 +9762,10 @@
     </row>
     <row r="68">
       <c r="A68" t="s" s="2">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" t="s" s="2">
@@ -9783,13 +9788,13 @@
         <v>81</v>
       </c>
       <c r="K68" t="s" s="2">
+        <v>448</v>
+      </c>
+      <c r="L68" t="s" s="2">
         <v>449</v>
       </c>
-      <c r="L68" t="s" s="2">
+      <c r="M68" t="s" s="2">
         <v>450</v>
-      </c>
-      <c r="M68" t="s" s="2">
-        <v>451</v>
       </c>
       <c r="N68" s="2"/>
       <c r="O68" s="2"/>
@@ -9840,7 +9845,7 @@
         <v>81</v>
       </c>
       <c r="AF68" t="s" s="2">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="AG68" t="s" s="2">
         <v>79</v>
@@ -9858,7 +9863,7 @@
         <v>81</v>
       </c>
       <c r="AL68" t="s" s="2">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="AM68" t="s" s="2">
         <v>81</v>
@@ -9869,10 +9874,10 @@
     </row>
     <row r="69">
       <c r="A69" t="s" s="2">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="B69" t="s" s="2">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" t="s" s="2">
@@ -9895,16 +9900,16 @@
         <v>81</v>
       </c>
       <c r="K69" t="s" s="2">
+        <v>453</v>
+      </c>
+      <c r="L69" t="s" s="2">
         <v>454</v>
       </c>
-      <c r="L69" t="s" s="2">
+      <c r="M69" t="s" s="2">
         <v>455</v>
       </c>
-      <c r="M69" t="s" s="2">
+      <c r="N69" t="s" s="2">
         <v>456</v>
-      </c>
-      <c r="N69" t="s" s="2">
-        <v>457</v>
       </c>
       <c r="O69" s="2"/>
       <c r="P69" t="s" s="2">
@@ -9954,7 +9959,7 @@
         <v>81</v>
       </c>
       <c r="AF69" t="s" s="2">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="AG69" t="s" s="2">
         <v>79</v>
@@ -9972,7 +9977,7 @@
         <v>81</v>
       </c>
       <c r="AL69" t="s" s="2">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="AM69" t="s" s="2">
         <v>81</v>
@@ -9983,10 +9988,10 @@
     </row>
     <row r="70">
       <c r="A70" t="s" s="2">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" t="s" s="2">
@@ -10012,13 +10017,13 @@
         <v>281</v>
       </c>
       <c r="L70" t="s" s="2">
+        <v>459</v>
+      </c>
+      <c r="M70" t="s" s="2">
         <v>460</v>
       </c>
-      <c r="M70" t="s" s="2">
+      <c r="N70" t="s" s="2">
         <v>461</v>
-      </c>
-      <c r="N70" t="s" s="2">
-        <v>462</v>
       </c>
       <c r="O70" s="2"/>
       <c r="P70" t="s" s="2">
@@ -10068,7 +10073,7 @@
         <v>81</v>
       </c>
       <c r="AF70" t="s" s="2">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="AG70" t="s" s="2">
         <v>79</v>
@@ -10086,7 +10091,7 @@
         <v>81</v>
       </c>
       <c r="AL70" t="s" s="2">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="AM70" t="s" s="2">
         <v>81</v>
@@ -10097,10 +10102,10 @@
     </row>
     <row r="71">
       <c r="A71" t="s" s="2">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="B71" t="s" s="2">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="C71" s="2"/>
       <c r="D71" t="s" s="2">
@@ -10209,10 +10214,10 @@
     </row>
     <row r="72">
       <c r="A72" t="s" s="2">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="B72" t="s" s="2">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" t="s" s="2">
@@ -10323,10 +10328,10 @@
     </row>
     <row r="73">
       <c r="A73" t="s" s="2">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="B73" t="s" s="2">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="C73" s="2"/>
       <c r="D73" t="s" s="2">
@@ -10439,10 +10444,10 @@
     </row>
     <row r="74">
       <c r="A74" t="s" s="2">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="B74" t="s" s="2">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" t="s" s="2">
@@ -10468,10 +10473,10 @@
         <v>210</v>
       </c>
       <c r="L74" t="s" s="2">
+        <v>467</v>
+      </c>
+      <c r="M74" t="s" s="2">
         <v>468</v>
-      </c>
-      <c r="M74" t="s" s="2">
-        <v>469</v>
       </c>
       <c r="N74" s="2"/>
       <c r="O74" s="2"/>
@@ -10522,7 +10527,7 @@
         <v>81</v>
       </c>
       <c r="AF74" t="s" s="2">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="AG74" t="s" s="2">
         <v>79</v>
@@ -10546,15 +10551,15 @@
         <v>81</v>
       </c>
       <c r="AN74" t="s" s="2">
-        <v>470</v>
+        <v>469</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="s" s="2">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="B75" t="s" s="2">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="C75" s="2"/>
       <c r="D75" t="s" s="2">
@@ -10663,10 +10668,10 @@
     </row>
     <row r="76">
       <c r="A76" t="s" s="2">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="B76" t="s" s="2">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C76" s="2"/>
       <c r="D76" t="s" s="2">
@@ -10777,10 +10782,10 @@
     </row>
     <row r="77">
       <c r="A77" t="s" s="2">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="B77" t="s" s="2">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="C77" s="2"/>
       <c r="D77" t="s" s="2">
@@ -10893,10 +10898,10 @@
     </row>
     <row r="78">
       <c r="A78" t="s" s="2">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="B78" t="s" s="2">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="C78" s="2"/>
       <c r="D78" t="s" s="2">
@@ -10925,7 +10930,7 @@
         <v>231</v>
       </c>
       <c r="M78" t="s" s="2">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="N78" t="s" s="2">
         <v>233</v>
@@ -11007,10 +11012,10 @@
     </row>
     <row r="79">
       <c r="A79" t="s" s="2">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="B79" t="s" s="2">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="C79" s="2"/>
       <c r="D79" t="s" s="2">
@@ -11039,7 +11044,7 @@
         <v>239</v>
       </c>
       <c r="M79" t="s" s="2">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="N79" t="s" s="2">
         <v>241</v>
@@ -11052,7 +11057,7 @@
       </c>
       <c r="Q79" s="2"/>
       <c r="R79" t="s" s="2">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="S79" t="s" s="2">
         <v>81</v>
@@ -11123,10 +11128,10 @@
     </row>
     <row r="80">
       <c r="A80" t="s" s="2">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B80" t="s" s="2">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="C80" s="2"/>
       <c r="D80" t="s" s="2">
@@ -11237,10 +11242,10 @@
     </row>
     <row r="81">
       <c r="A81" t="s" s="2">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="B81" t="s" s="2">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="C81" s="2"/>
       <c r="D81" t="s" s="2">
@@ -11349,10 +11354,10 @@
     </row>
     <row r="82">
       <c r="A82" t="s" s="2">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="B82" t="s" s="2">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="C82" s="2"/>
       <c r="D82" t="s" s="2">
@@ -11463,10 +11468,10 @@
     </row>
     <row r="83">
       <c r="A83" t="s" s="2">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="B83" t="s" s="2">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="C83" s="2"/>
       <c r="D83" t="s" s="2">
@@ -11489,13 +11494,13 @@
         <v>81</v>
       </c>
       <c r="K83" t="s" s="2">
+        <v>482</v>
+      </c>
+      <c r="L83" t="s" s="2">
         <v>483</v>
       </c>
-      <c r="L83" t="s" s="2">
+      <c r="M83" t="s" s="2">
         <v>484</v>
-      </c>
-      <c r="M83" t="s" s="2">
-        <v>485</v>
       </c>
       <c r="N83" s="2"/>
       <c r="O83" s="2"/>
@@ -11546,7 +11551,7 @@
         <v>81</v>
       </c>
       <c r="AF83" t="s" s="2">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="AG83" t="s" s="2">
         <v>79</v>
@@ -11564,7 +11569,7 @@
         <v>81</v>
       </c>
       <c r="AL83" t="s" s="2">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="AM83" t="s" s="2">
         <v>81</v>
@@ -11575,10 +11580,10 @@
     </row>
     <row r="84">
       <c r="A84" t="s" s="2">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="B84" t="s" s="2">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C84" s="2"/>
       <c r="D84" t="s" s="2">
@@ -11604,10 +11609,10 @@
         <v>230</v>
       </c>
       <c r="L84" t="s" s="2">
+        <v>487</v>
+      </c>
+      <c r="M84" t="s" s="2">
         <v>488</v>
-      </c>
-      <c r="M84" t="s" s="2">
-        <v>489</v>
       </c>
       <c r="N84" s="2"/>
       <c r="O84" s="2"/>
@@ -11638,7 +11643,7 @@
       </c>
       <c r="Y84" s="2"/>
       <c r="Z84" t="s" s="2">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="AA84" t="s" s="2">
         <v>81</v>
@@ -11656,7 +11661,7 @@
         <v>81</v>
       </c>
       <c r="AF84" t="s" s="2">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="AG84" t="s" s="2">
         <v>79</v>
@@ -11674,21 +11679,21 @@
         <v>81</v>
       </c>
       <c r="AL84" t="s" s="2">
+        <v>490</v>
+      </c>
+      <c r="AM84" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN84" t="s" s="2">
         <v>491</v>
-      </c>
-      <c r="AM84" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AN84" t="s" s="2">
-        <v>492</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="s" s="2">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="B85" t="s" s="2">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="C85" s="2"/>
       <c r="D85" t="s" s="2">
@@ -11714,10 +11719,10 @@
         <v>230</v>
       </c>
       <c r="L85" t="s" s="2">
+        <v>493</v>
+      </c>
+      <c r="M85" t="s" s="2">
         <v>494</v>
-      </c>
-      <c r="M85" t="s" s="2">
-        <v>495</v>
       </c>
       <c r="N85" s="2"/>
       <c r="O85" s="2"/>
@@ -11747,11 +11752,11 @@
         <v>160</v>
       </c>
       <c r="Y85" t="s" s="2">
+        <v>495</v>
+      </c>
+      <c r="Z85" t="s" s="2">
         <v>496</v>
       </c>
-      <c r="Z85" t="s" s="2">
-        <v>497</v>
-      </c>
       <c r="AA85" t="s" s="2">
         <v>81</v>
       </c>
@@ -11768,7 +11773,7 @@
         <v>81</v>
       </c>
       <c r="AF85" t="s" s="2">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="AG85" t="s" s="2">
         <v>79</v>
@@ -11792,15 +11797,15 @@
         <v>81</v>
       </c>
       <c r="AN85" t="s" s="2">
-        <v>498</v>
+        <v>497</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="s" s="2">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B86" t="s" s="2">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="C86" s="2"/>
       <c r="D86" t="s" s="2">
@@ -11826,16 +11831,16 @@
         <v>230</v>
       </c>
       <c r="L86" t="s" s="2">
+        <v>499</v>
+      </c>
+      <c r="M86" t="s" s="2">
         <v>500</v>
       </c>
-      <c r="M86" t="s" s="2">
+      <c r="N86" t="s" s="2">
         <v>501</v>
       </c>
-      <c r="N86" t="s" s="2">
+      <c r="O86" t="s" s="2">
         <v>502</v>
-      </c>
-      <c r="O86" t="s" s="2">
-        <v>503</v>
       </c>
       <c r="P86" t="s" s="2">
         <v>81</v>
@@ -11863,11 +11868,11 @@
         <v>160</v>
       </c>
       <c r="Y86" t="s" s="2">
+        <v>503</v>
+      </c>
+      <c r="Z86" t="s" s="2">
         <v>504</v>
       </c>
-      <c r="Z86" t="s" s="2">
-        <v>505</v>
-      </c>
       <c r="AA86" t="s" s="2">
         <v>81</v>
       </c>
@@ -11884,7 +11889,7 @@
         <v>81</v>
       </c>
       <c r="AF86" t="s" s="2">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="AG86" t="s" s="2">
         <v>79</v>
@@ -11902,21 +11907,21 @@
         <v>81</v>
       </c>
       <c r="AL86" t="s" s="2">
+        <v>505</v>
+      </c>
+      <c r="AM86" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN86" t="s" s="2">
         <v>506</v>
-      </c>
-      <c r="AM86" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AN86" t="s" s="2">
-        <v>507</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="s" s="2">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="B87" t="s" s="2">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="C87" s="2"/>
       <c r="D87" t="s" s="2">
@@ -11942,10 +11947,10 @@
         <v>230</v>
       </c>
       <c r="L87" t="s" s="2">
+        <v>508</v>
+      </c>
+      <c r="M87" t="s" s="2">
         <v>509</v>
-      </c>
-      <c r="M87" t="s" s="2">
-        <v>510</v>
       </c>
       <c r="N87" s="2"/>
       <c r="O87" s="2"/>
@@ -11975,11 +11980,11 @@
         <v>174</v>
       </c>
       <c r="Y87" t="s" s="2">
+        <v>510</v>
+      </c>
+      <c r="Z87" t="s" s="2">
         <v>511</v>
       </c>
-      <c r="Z87" t="s" s="2">
-        <v>512</v>
-      </c>
       <c r="AA87" t="s" s="2">
         <v>81</v>
       </c>
@@ -11996,7 +12001,7 @@
         <v>81</v>
       </c>
       <c r="AF87" t="s" s="2">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="AG87" t="s" s="2">
         <v>79</v>
@@ -12014,21 +12019,21 @@
         <v>81</v>
       </c>
       <c r="AL87" t="s" s="2">
+        <v>512</v>
+      </c>
+      <c r="AM87" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN87" t="s" s="2">
         <v>513</v>
-      </c>
-      <c r="AM87" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AN87" t="s" s="2">
-        <v>514</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="s" s="2">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="B88" t="s" s="2">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="C88" s="2"/>
       <c r="D88" t="s" s="2">
@@ -12054,10 +12059,10 @@
         <v>230</v>
       </c>
       <c r="L88" t="s" s="2">
+        <v>515</v>
+      </c>
+      <c r="M88" t="s" s="2">
         <v>516</v>
-      </c>
-      <c r="M88" t="s" s="2">
-        <v>517</v>
       </c>
       <c r="N88" s="2"/>
       <c r="O88" s="2"/>
@@ -12087,11 +12092,11 @@
         <v>174</v>
       </c>
       <c r="Y88" t="s" s="2">
+        <v>517</v>
+      </c>
+      <c r="Z88" t="s" s="2">
         <v>518</v>
       </c>
-      <c r="Z88" t="s" s="2">
-        <v>519</v>
-      </c>
       <c r="AA88" t="s" s="2">
         <v>81</v>
       </c>
@@ -12108,7 +12113,7 @@
         <v>81</v>
       </c>
       <c r="AF88" t="s" s="2">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="AG88" t="s" s="2">
         <v>79</v>
@@ -12126,21 +12131,21 @@
         <v>81</v>
       </c>
       <c r="AL88" t="s" s="2">
+        <v>519</v>
+      </c>
+      <c r="AM88" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN88" t="s" s="2">
         <v>520</v>
-      </c>
-      <c r="AM88" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AN88" t="s" s="2">
-        <v>521</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="s" s="2">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B89" t="s" s="2">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="C89" s="2"/>
       <c r="D89" t="s" s="2">
@@ -12163,13 +12168,13 @@
         <v>81</v>
       </c>
       <c r="K89" t="s" s="2">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="L89" t="s" s="2">
+        <v>522</v>
+      </c>
+      <c r="M89" t="s" s="2">
         <v>523</v>
-      </c>
-      <c r="M89" t="s" s="2">
-        <v>524</v>
       </c>
       <c r="N89" s="2"/>
       <c r="O89" s="2"/>
@@ -12220,7 +12225,7 @@
         <v>81</v>
       </c>
       <c r="AF89" t="s" s="2">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="AG89" t="s" s="2">
         <v>79</v>
@@ -12238,21 +12243,21 @@
         <v>81</v>
       </c>
       <c r="AL89" t="s" s="2">
+        <v>524</v>
+      </c>
+      <c r="AM89" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN89" t="s" s="2">
         <v>525</v>
-      </c>
-      <c r="AM89" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AN89" t="s" s="2">
-        <v>526</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="s" s="2">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="B90" t="s" s="2">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="C90" s="2"/>
       <c r="D90" t="s" s="2">
@@ -12278,10 +12283,10 @@
         <v>230</v>
       </c>
       <c r="L90" t="s" s="2">
+        <v>527</v>
+      </c>
+      <c r="M90" t="s" s="2">
         <v>528</v>
-      </c>
-      <c r="M90" t="s" s="2">
-        <v>529</v>
       </c>
       <c r="N90" s="2"/>
       <c r="O90" s="2"/>
@@ -12312,7 +12317,7 @@
       </c>
       <c r="Y90" s="2"/>
       <c r="Z90" t="s" s="2">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="AA90" t="s" s="2">
         <v>81</v>
@@ -12330,7 +12335,7 @@
         <v>81</v>
       </c>
       <c r="AF90" t="s" s="2">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="AG90" t="s" s="2">
         <v>79</v>
@@ -12348,21 +12353,21 @@
         <v>81</v>
       </c>
       <c r="AL90" t="s" s="2">
+        <v>530</v>
+      </c>
+      <c r="AM90" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN90" t="s" s="2">
         <v>531</v>
-      </c>
-      <c r="AM90" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AN90" t="s" s="2">
-        <v>532</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="s" s="2">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="B91" t="s" s="2">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="C91" s="2"/>
       <c r="D91" t="s" s="2">
@@ -12388,13 +12393,13 @@
         <v>281</v>
       </c>
       <c r="L91" t="s" s="2">
+        <v>533</v>
+      </c>
+      <c r="M91" t="s" s="2">
         <v>534</v>
       </c>
-      <c r="M91" t="s" s="2">
+      <c r="N91" t="s" s="2">
         <v>535</v>
-      </c>
-      <c r="N91" t="s" s="2">
-        <v>536</v>
       </c>
       <c r="O91" s="2"/>
       <c r="P91" t="s" s="2">
@@ -12444,7 +12449,7 @@
         <v>81</v>
       </c>
       <c r="AF91" t="s" s="2">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="AG91" t="s" s="2">
         <v>79</v>
@@ -12462,7 +12467,7 @@
         <v>81</v>
       </c>
       <c r="AL91" t="s" s="2">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="AM91" t="s" s="2">
         <v>81</v>
@@ -12473,10 +12478,10 @@
     </row>
     <row r="92">
       <c r="A92" t="s" s="2">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="B92" t="s" s="2">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="C92" s="2"/>
       <c r="D92" t="s" s="2">
@@ -12585,10 +12590,10 @@
     </row>
     <row r="93">
       <c r="A93" t="s" s="2">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="B93" t="s" s="2">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="C93" s="2"/>
       <c r="D93" t="s" s="2">
@@ -12699,10 +12704,10 @@
     </row>
     <row r="94">
       <c r="A94" t="s" s="2">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="B94" t="s" s="2">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="C94" s="2"/>
       <c r="D94" t="s" s="2">
@@ -12815,10 +12820,10 @@
     </row>
     <row r="95">
       <c r="A95" t="s" s="2">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B95" t="s" s="2">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="C95" s="2"/>
       <c r="D95" t="s" s="2">
@@ -12841,13 +12846,13 @@
         <v>81</v>
       </c>
       <c r="K95" t="s" s="2">
+        <v>541</v>
+      </c>
+      <c r="L95" t="s" s="2">
         <v>542</v>
       </c>
-      <c r="L95" t="s" s="2">
+      <c r="M95" t="s" s="2">
         <v>543</v>
-      </c>
-      <c r="M95" t="s" s="2">
-        <v>544</v>
       </c>
       <c r="N95" s="2"/>
       <c r="O95" s="2"/>
@@ -12898,7 +12903,7 @@
         <v>81</v>
       </c>
       <c r="AF95" t="s" s="2">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="AG95" t="s" s="2">
         <v>89</v>
@@ -12913,24 +12918,24 @@
         <v>101</v>
       </c>
       <c r="AK95" t="s" s="2">
+        <v>544</v>
+      </c>
+      <c r="AL95" t="s" s="2">
+        <v>389</v>
+      </c>
+      <c r="AM95" t="s" s="2">
         <v>545</v>
       </c>
-      <c r="AL95" t="s" s="2">
-        <v>390</v>
-      </c>
-      <c r="AM95" t="s" s="2">
+      <c r="AN95" t="s" s="2">
         <v>546</v>
-      </c>
-      <c r="AN95" t="s" s="2">
-        <v>547</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="s" s="2">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="B96" t="s" s="2">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
@@ -12956,13 +12961,13 @@
         <v>170</v>
       </c>
       <c r="L96" t="s" s="2">
+        <v>548</v>
+      </c>
+      <c r="M96" t="s" s="2">
         <v>549</v>
       </c>
-      <c r="M96" t="s" s="2">
+      <c r="N96" t="s" s="2">
         <v>550</v>
-      </c>
-      <c r="N96" t="s" s="2">
-        <v>551</v>
       </c>
       <c r="O96" s="2"/>
       <c r="P96" t="s" s="2">
@@ -12991,11 +12996,11 @@
         <v>224</v>
       </c>
       <c r="Y96" t="s" s="2">
+        <v>551</v>
+      </c>
+      <c r="Z96" t="s" s="2">
         <v>552</v>
       </c>
-      <c r="Z96" t="s" s="2">
-        <v>553</v>
-      </c>
       <c r="AA96" t="s" s="2">
         <v>81</v>
       </c>
@@ -13012,7 +13017,7 @@
         <v>81</v>
       </c>
       <c r="AF96" t="s" s="2">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="AG96" t="s" s="2">
         <v>79</v>
@@ -13030,7 +13035,7 @@
         <v>81</v>
       </c>
       <c r="AL96" t="s" s="2">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="AM96" t="s" s="2">
         <v>81</v>
@@ -13041,10 +13046,10 @@
     </row>
     <row r="97">
       <c r="A97" t="s" s="2">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="B97" t="s" s="2">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="C97" s="2"/>
       <c r="D97" t="s" s="2">
@@ -13070,13 +13075,13 @@
         <v>230</v>
       </c>
       <c r="L97" t="s" s="2">
+        <v>555</v>
+      </c>
+      <c r="M97" t="s" s="2">
         <v>556</v>
       </c>
-      <c r="M97" t="s" s="2">
+      <c r="N97" t="s" s="2">
         <v>557</v>
-      </c>
-      <c r="N97" t="s" s="2">
-        <v>558</v>
       </c>
       <c r="O97" s="2"/>
       <c r="P97" t="s" s="2">
@@ -13106,7 +13111,7 @@
       </c>
       <c r="Y97" s="2"/>
       <c r="Z97" t="s" s="2">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="AA97" t="s" s="2">
         <v>81</v>
@@ -13124,7 +13129,7 @@
         <v>81</v>
       </c>
       <c r="AF97" t="s" s="2">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="AG97" t="s" s="2">
         <v>79</v>
@@ -13153,10 +13158,10 @@
     </row>
     <row r="98">
       <c r="A98" t="s" s="2">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="B98" t="s" s="2">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="C98" s="2"/>
       <c r="D98" t="s" s="2">
@@ -13182,10 +13187,10 @@
         <v>256</v>
       </c>
       <c r="L98" t="s" s="2">
+        <v>560</v>
+      </c>
+      <c r="M98" t="s" s="2">
         <v>561</v>
-      </c>
-      <c r="M98" t="s" s="2">
-        <v>562</v>
       </c>
       <c r="N98" s="2"/>
       <c r="O98" s="2"/>
@@ -13236,7 +13241,7 @@
         <v>81</v>
       </c>
       <c r="AF98" t="s" s="2">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="AG98" t="s" s="2">
         <v>79</v>
@@ -13254,7 +13259,7 @@
         <v>81</v>
       </c>
       <c r="AL98" t="s" s="2">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="AM98" t="s" s="2">
         <v>81</v>
@@ -13265,10 +13270,10 @@
     </row>
     <row r="99">
       <c r="A99" t="s" s="2">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="B99" t="s" s="2">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="C99" s="2"/>
       <c r="D99" t="s" s="2">
@@ -13294,10 +13299,10 @@
         <v>263</v>
       </c>
       <c r="L99" t="s" s="2">
+        <v>563</v>
+      </c>
+      <c r="M99" t="s" s="2">
         <v>564</v>
-      </c>
-      <c r="M99" t="s" s="2">
-        <v>565</v>
       </c>
       <c r="N99" s="2"/>
       <c r="O99" s="2"/>
@@ -13348,7 +13353,7 @@
         <v>81</v>
       </c>
       <c r="AF99" t="s" s="2">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="AG99" t="s" s="2">
         <v>79</v>
@@ -13363,24 +13368,24 @@
         <v>101</v>
       </c>
       <c r="AK99" t="s" s="2">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="AL99" t="s" s="2">
+        <v>565</v>
+      </c>
+      <c r="AM99" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AN99" t="s" s="2">
         <v>566</v>
-      </c>
-      <c r="AM99" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AN99" t="s" s="2">
-        <v>567</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="s" s="2">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="B100" t="s" s="2">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="C100" s="2"/>
       <c r="D100" t="s" s="2">
@@ -13403,16 +13408,16 @@
         <v>81</v>
       </c>
       <c r="K100" t="s" s="2">
+        <v>568</v>
+      </c>
+      <c r="L100" t="s" s="2">
         <v>569</v>
       </c>
-      <c r="L100" t="s" s="2">
+      <c r="M100" t="s" s="2">
         <v>570</v>
       </c>
-      <c r="M100" t="s" s="2">
+      <c r="N100" t="s" s="2">
         <v>571</v>
-      </c>
-      <c r="N100" t="s" s="2">
-        <v>572</v>
       </c>
       <c r="O100" s="2"/>
       <c r="P100" t="s" s="2">
@@ -13462,7 +13467,7 @@
         <v>81</v>
       </c>
       <c r="AF100" t="s" s="2">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="AG100" t="s" s="2">
         <v>79</v>
@@ -13477,10 +13482,10 @@
         <v>101</v>
       </c>
       <c r="AK100" t="s" s="2">
+        <v>572</v>
+      </c>
+      <c r="AL100" t="s" s="2">
         <v>573</v>
-      </c>
-      <c r="AL100" t="s" s="2">
-        <v>574</v>
       </c>
       <c r="AM100" t="s" s="2">
         <v>81</v>

</xml_diff>

<commit_message>
Remove commented-out FRActorExtension participant constraints
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> b739922ccd7998ba51709aade89054ea0313b6fd
</commit_message>
<xml_diff>
--- a/nr-doc-core-encounter/ig/StructureDefinition-fr-core-encounter.xlsx
+++ b/nr-doc-core-encounter/ig/StructureDefinition-fr-core-encounter.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-21T11:52:46+00:00</t>
+    <t>2026-07-21T11:54:41+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -943,13 +943,7 @@
     <t>Encounter.class</t>
   </si>
   <si>
-    <t>Type de rencontre (codes HL7 ActEncounterCode ou codes spécifiques aux cas d'usages)
-Exemples de codes les plus courants (http://terminology.hl7.org/CodeSystem/v3-ActCode) :
-- ACUTE : Inpatient acute
-- NONAC : Inpatient non acute
-- PRENC : Pre-admission
-- SS : Short stay
-- VR : Virtual</t>
+    <t>Type de rencontre (codes HL7 ActEncounterCode ou codes spécifiques aux cas d'usages) — exemples les plus courants (v3-ActCode) : ACUTE (Inpatient acute), NONAC (Inpatient non acute), PRENC (Pre-admission), SS (Short stay), VR (Virtual)</t>
   </si>
   <si>
     <t>Concepts representing classification of patient encounter such as ambulatory (outpatient), inpatient, emergency, home health or others due to local variations.</t>
@@ -1051,9 +1045,7 @@
     <t>Encounter.priority</t>
   </si>
   <si>
-    <t>Si la rencontre est prévue non confirmée et qu'une confirmation est attendue :
-code='CS', display='callback for scheduling'
-Sinon, l'élément 'priority' n'est pas fourni.</t>
+    <t>Si la rencontre est prévue non confirmée et qu'une confirmation est attendue : code='CS', display='callback for scheduling'. Sinon, l'élément 'priority' n'est pas fourni.</t>
   </si>
   <si>
     <t>Indicates the urgency of the encounter.</t>
@@ -1261,9 +1253,7 @@
     <t>Encounter.period</t>
   </si>
   <si>
-    <t>Date début et fin de la rencontre
-Si la rencontre est réalisée ou planifiée : la date est obligatoire.
-Si la rencontre est prévue non confirmée : la date est facultative.</t>
+    <t>Date début et fin de la rencontre. Si la rencontre est réalisée ou planifiée : la date est obligatoire. Si la rencontre est prévue non confirmée : la date est facultative.</t>
   </si>
   <si>
     <t>The start and end time of the encounter.</t>
@@ -1658,8 +1648,7 @@
     <t>Encounter.hospitalization.dischargeDisposition</t>
   </si>
   <si>
-    <t>Modalité de sortie du patient lors de la rencontre:
-Valeur provenant du jdv-modalite-sortie-cisis ou autre JDV spécifique au volet</t>
+    <t>Modalité de sortie du patient lors de la rencontre : valeur provenant du jdv-modalite-sortie-cisis ou autre JDV spécifique au volet</t>
   </si>
   <si>
     <t>Category or kind of location after discharge.</t>

</xml_diff>

<commit_message>
Update dischargeDisposition short description de9d6c0f4fce70b6c31a999f0b6547fe02751e89
</commit_message>
<xml_diff>
--- a/nr-doc-core-encounter/ig/StructureDefinition-fr-core-encounter.xlsx
+++ b/nr-doc-core-encounter/ig/StructureDefinition-fr-core-encounter.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-27T13:42:38+00:00</t>
+    <t>2026-07-27T13:52:49+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1654,7 +1654,7 @@
     <t>Encounter.hospitalization.dischargeDisposition</t>
   </si>
   <si>
-    <t>Modalité de sortie du patient lors de la rencontre : valeur provenant du jdv-modalite-sortie-cisis ou autre JDV spécifique au volet</t>
+    <t>Modalité de sortie du patient lors de la rencontre.</t>
   </si>
   <si>
     <t>Category or kind of location after discharge.</t>

</xml_diff>

<commit_message>
fix: retrait du binding hospitalization.dischargeDisposition vers FRCoreValueSetEncounterDischargeDisposition
Le ValueSet mélangeait des codes ne correspondant pas forcément à une simple
catégorie de lieu et pouvant être cumulables (ex: fugue + Home) alors que la
cardinalité de l'élément est 0..1, source d'ambiguïté pour l'implémentation.
Retrait du ValueSet, du CodeSystem associé (FRCoreCodeSystemCirconstancesSortie)
et de leurs traductions, en attendant un travail complémentaire au GT IHE PAM en FHIR.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> edd7490f6acc8a82b4b7fff8666cf2f6dd6e513c
</commit_message>
<xml_diff>
--- a/nr-doc-core-encounter/ig/StructureDefinition-fr-core-encounter.xlsx
+++ b/nr-doc-core-encounter/ig/StructureDefinition-fr-core-encounter.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3608" uniqueCount="576">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3609" uniqueCount="577">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-27T13:55:37+00:00</t>
+    <t>2026-07-27T16:09:25+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1660,7 +1660,10 @@
     <t>Category or kind of location after discharge.</t>
   </si>
   <si>
-    <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-encounter-discharge-disposition|2.2.0</t>
+    <t>Discharge Disposition.</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/ValueSet/encounter-discharge-disposition|4.0.1</t>
   </si>
   <si>
     <t>.dischargeDispositionCode</t>
@@ -12310,9 +12313,11 @@
       <c r="X90" t="s" s="2">
         <v>160</v>
       </c>
-      <c r="Y90" s="2"/>
+      <c r="Y90" t="s" s="2">
+        <v>531</v>
+      </c>
       <c r="Z90" t="s" s="2">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="AA90" t="s" s="2">
         <v>81</v>
@@ -12348,21 +12353,21 @@
         <v>81</v>
       </c>
       <c r="AL90" t="s" s="2">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="AM90" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AN90" t="s" s="2">
-        <v>533</v>
+        <v>534</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="s" s="2">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="B91" t="s" s="2">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="C91" s="2"/>
       <c r="D91" t="s" s="2">
@@ -12388,13 +12393,13 @@
         <v>281</v>
       </c>
       <c r="L91" t="s" s="2">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="M91" t="s" s="2">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="N91" t="s" s="2">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="O91" s="2"/>
       <c r="P91" t="s" s="2">
@@ -12444,7 +12449,7 @@
         <v>81</v>
       </c>
       <c r="AF91" t="s" s="2">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="AG91" t="s" s="2">
         <v>79</v>
@@ -12462,7 +12467,7 @@
         <v>81</v>
       </c>
       <c r="AL91" t="s" s="2">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="AM91" t="s" s="2">
         <v>81</v>
@@ -12473,10 +12478,10 @@
     </row>
     <row r="92">
       <c r="A92" t="s" s="2">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="B92" t="s" s="2">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="C92" s="2"/>
       <c r="D92" t="s" s="2">
@@ -12585,10 +12590,10 @@
     </row>
     <row r="93">
       <c r="A93" t="s" s="2">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="B93" t="s" s="2">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="C93" s="2"/>
       <c r="D93" t="s" s="2">
@@ -12699,10 +12704,10 @@
     </row>
     <row r="94">
       <c r="A94" t="s" s="2">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="B94" t="s" s="2">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="C94" s="2"/>
       <c r="D94" t="s" s="2">
@@ -12815,10 +12820,10 @@
     </row>
     <row r="95">
       <c r="A95" t="s" s="2">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="B95" t="s" s="2">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="C95" s="2"/>
       <c r="D95" t="s" s="2">
@@ -12841,13 +12846,13 @@
         <v>81</v>
       </c>
       <c r="K95" t="s" s="2">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="L95" t="s" s="2">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="M95" t="s" s="2">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="N95" s="2"/>
       <c r="O95" s="2"/>
@@ -12898,7 +12903,7 @@
         <v>81</v>
       </c>
       <c r="AF95" t="s" s="2">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="AG95" t="s" s="2">
         <v>89</v>
@@ -12913,24 +12918,24 @@
         <v>101</v>
       </c>
       <c r="AK95" t="s" s="2">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="AL95" t="s" s="2">
         <v>390</v>
       </c>
       <c r="AM95" t="s" s="2">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="AN95" t="s" s="2">
-        <v>548</v>
+        <v>549</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="s" s="2">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="B96" t="s" s="2">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="C96" s="2"/>
       <c r="D96" t="s" s="2">
@@ -12956,13 +12961,13 @@
         <v>170</v>
       </c>
       <c r="L96" t="s" s="2">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="M96" t="s" s="2">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="N96" t="s" s="2">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="O96" s="2"/>
       <c r="P96" t="s" s="2">
@@ -12991,10 +12996,10 @@
         <v>224</v>
       </c>
       <c r="Y96" t="s" s="2">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="Z96" t="s" s="2">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="AA96" t="s" s="2">
         <v>81</v>
@@ -13012,7 +13017,7 @@
         <v>81</v>
       </c>
       <c r="AF96" t="s" s="2">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="AG96" t="s" s="2">
         <v>79</v>
@@ -13030,7 +13035,7 @@
         <v>81</v>
       </c>
       <c r="AL96" t="s" s="2">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="AM96" t="s" s="2">
         <v>81</v>
@@ -13041,10 +13046,10 @@
     </row>
     <row r="97">
       <c r="A97" t="s" s="2">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="B97" t="s" s="2">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="C97" s="2"/>
       <c r="D97" t="s" s="2">
@@ -13070,13 +13075,13 @@
         <v>230</v>
       </c>
       <c r="L97" t="s" s="2">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="M97" t="s" s="2">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="N97" t="s" s="2">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="O97" s="2"/>
       <c r="P97" t="s" s="2">
@@ -13106,7 +13111,7 @@
       </c>
       <c r="Y97" s="2"/>
       <c r="Z97" t="s" s="2">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="AA97" t="s" s="2">
         <v>81</v>
@@ -13124,7 +13129,7 @@
         <v>81</v>
       </c>
       <c r="AF97" t="s" s="2">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="AG97" t="s" s="2">
         <v>79</v>
@@ -13153,10 +13158,10 @@
     </row>
     <row r="98">
       <c r="A98" t="s" s="2">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="B98" t="s" s="2">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="C98" s="2"/>
       <c r="D98" t="s" s="2">
@@ -13182,10 +13187,10 @@
         <v>256</v>
       </c>
       <c r="L98" t="s" s="2">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="M98" t="s" s="2">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="N98" s="2"/>
       <c r="O98" s="2"/>
@@ -13236,7 +13241,7 @@
         <v>81</v>
       </c>
       <c r="AF98" t="s" s="2">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="AG98" t="s" s="2">
         <v>79</v>
@@ -13265,10 +13270,10 @@
     </row>
     <row r="99">
       <c r="A99" t="s" s="2">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="B99" t="s" s="2">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="C99" s="2"/>
       <c r="D99" t="s" s="2">
@@ -13294,10 +13299,10 @@
         <v>263</v>
       </c>
       <c r="L99" t="s" s="2">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="M99" t="s" s="2">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="N99" s="2"/>
       <c r="O99" s="2"/>
@@ -13348,7 +13353,7 @@
         <v>81</v>
       </c>
       <c r="AF99" t="s" s="2">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="AG99" t="s" s="2">
         <v>79</v>
@@ -13366,21 +13371,21 @@
         <v>389</v>
       </c>
       <c r="AL99" t="s" s="2">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="AM99" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AN99" t="s" s="2">
-        <v>568</v>
+        <v>569</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="s" s="2">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="B100" t="s" s="2">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="C100" s="2"/>
       <c r="D100" t="s" s="2">
@@ -13403,16 +13408,16 @@
         <v>81</v>
       </c>
       <c r="K100" t="s" s="2">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="L100" t="s" s="2">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="M100" t="s" s="2">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="N100" t="s" s="2">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="O100" s="2"/>
       <c r="P100" t="s" s="2">
@@ -13462,7 +13467,7 @@
         <v>81</v>
       </c>
       <c r="AF100" t="s" s="2">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="AG100" t="s" s="2">
         <v>79</v>
@@ -13477,10 +13482,10 @@
         <v>101</v>
       </c>
       <c r="AK100" t="s" s="2">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="AL100" t="s" s="2">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="AM100" t="s" s="2">
         <v>81</v>

</xml_diff>

<commit_message>
Update subject reference options in FRCoreEncounterProfile 192130c946bbf9fdd21bff19b351f8faece1a3c8
</commit_message>
<xml_diff>
--- a/nr-doc-core-encounter/ig/StructureDefinition-fr-core-encounter.xlsx
+++ b/nr-doc-core-encounter/ig/StructureDefinition-fr-core-encounter.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-27T16:09:25+00:00</t>
+    <t>2026-07-28T08:44:28+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1073,7 +1073,7 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-patient|2.2.0|Group|4.0.1)
+    <t xml:space="preserve">Reference(https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-patient-ins|2.2.0|https://hl7.fr/ig/fhir/core/StructureDefinition/fr-core-patient|2.2.0|Group|4.0.1)
 </t>
   </si>
   <si>
@@ -2123,7 +2123,7 @@
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="117.0625" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="124.91015625" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>

</xml_diff>